<commit_message>
run several iterations of new best
</commit_message>
<xml_diff>
--- a/Deep_Learning/combined.xlsx
+++ b/Deep_Learning/combined.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bmanderson\Desktop\Modular_Projects\Liver_Disease_Ablation_Segmentation\Deep_Learning\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Modular_Projects\Liver_Disease_Ablation_Segmentation\Deep_Learning\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -463,7 +463,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:U23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -602,7 +601,7 @@
         <v>0.83398008346557617</v>
       </c>
     </row>
-    <row r="3" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>174</v>
       </c>
@@ -732,7 +731,7 @@
         <v>0.8223036527633667</v>
       </c>
     </row>
-    <row r="5" spans="1:21" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>176</v>
       </c>
@@ -1969,30 +1968,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:U23">
-    <filterColumn colId="0">
-      <filters>
-        <filter val="177"/>
-        <filter val="178"/>
-        <filter val="179"/>
-        <filter val="180"/>
-        <filter val="181"/>
-        <filter val="182"/>
-        <filter val="183"/>
-        <filter val="184"/>
-        <filter val="185"/>
-        <filter val="186"/>
-        <filter val="187"/>
-        <filter val="188"/>
-        <filter val="189"/>
-        <filter val="190"/>
-        <filter val="191"/>
-        <filter val="192"/>
-        <filter val="193"/>
-        <filter val="194"/>
-        <filter val="195"/>
-        <filter val="196"/>
-      </filters>
-    </filterColumn>
     <sortState ref="A2:U23">
       <sortCondition ref="S1"/>
     </sortState>

</xml_diff>